<commit_message>
html and css separate files created
</commit_message>
<xml_diff>
--- a/Few_shot_examples.xlsx
+++ b/Few_shot_examples.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC26\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\vs code\RelevanceIQ  - FTO - Updated-UI-Reasoning - Copy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8404FB05-0BD3-47F6-A8F3-78C9AC32DE04}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D2071AD-3593-4A1F-B3CC-61B960EF73EB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -19,10 +19,10 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'By Source'!$A$1:$D$8</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Golden Dataset'!$A$1:$H$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Golden Dataset'!$A$1:$G$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Overall Distribution'!$A$1:$B$5</definedName>
   </definedNames>
-  <calcPr calcId="191029" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
@@ -32,15 +32,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="75">
   <si>
     <t>Product Description</t>
   </si>
   <si>
     <t>Publication Number</t>
-  </si>
-  <si>
-    <t>title</t>
   </si>
   <si>
     <t>Relevance Rating</t>
@@ -155,103 +152,13 @@
  10. According to the grass mowing robot described in claim 9, the invention is characterized in that: the lower seat body (12) is provided with point-shaped or strip-shaped anti-skid protrusions (121).</t>
   </si>
   <si>
-    <t>A lawn mower grass-comb assembly comprising front, middle, and rear grass combs integrated into a common hardware component. The front grass comb is wider than the rear grass comb, while both extend to the same lower height. The mid-grass comb extends to a comparatively higher position with a shorter downward extension, creating a differentiated comb configuration designed to guide and manage grass around different portions of the mower during operation.</t>
-  </si>
-  <si>
-    <t>US20260198411A1</t>
-  </si>
-  <si>
-    <t>Robotic lawn mower</t>
-  </si>
-  <si>
-    <t>A robotic lawn mower may be adapted for a forward travelling direction and a reverse travelling direction and include a body that has a frontmost end adapted to face the forward travelling direction and ground during normal operation, and a rearmost end adapted to face the reverse travelling direction and ground during normal operation. The robotic lawn mower includes a pair of drive wheels, a further wheel, and a rotatable grass cutting disc having a disc rotation axle. The robotic lawn mower includes a mat arrangement that includes a mat positioned between the frontmost end and the rearmost end, having a mainly longitudinally running first edge that runs mainly across the forward running direction and is adapted to be the part of the mat that is closest to ground during normal operation. The mat arrangement includes a mat attachment arrangement connecting the mat to the body in a movable manner.</t>
-  </si>
-  <si>
-    <t>1. A robotic lawn mower adapted for a forward travelling direction and a reverse travelling direction and comprising a body that has a frontmost end that is adapted to face the forward travelling direction and ground during normal operation, and a rearmost end that is adapted to face the reverse travelling direction and ground during normal operation, the robotic lawn mower further comprising at least one pair of drive wheels, at least one further wheel, and at least one rotatable grass cutting disc having a disc rotation axle, wherein the robotic lawn mower further comprises a mat arrangement that in turn comprises a mat that is positioned between the frontmost end and the rearmost end, having a mainly longitudinally running first edge that runs mainly across the forward running direction and is adapted to be the part of the mat that is closest to ground during normal operation, wherein the mat arrangement comprises a mat attachment arrangement that connects the mat to the body in a movable manner.</t>
-  </si>
-  <si>
-    <t>1. A robotic lawn mower adapted for a forward travelling direction and a reverse travelling direction and comprising a body that has a frontmost end that is adapted to face the forward travelling direction and ground during normal operation, and a rearmost end that is adapted to face the reverse travelling direction and ground during normal operation, the robotic lawn mower further comprising at least one pair of drive wheels, at least one further wheel, and at least one rotatable grass cutting disc having a disc rotation axle, wherein the robotic lawn mower further comprises a mat arrangement that in turn comprises a mat that is positioned between the frontmost end and the rearmost end, having a mainly longitudinally running first edge that runs mainly across the forward running direction and is adapted to be the part of the mat that is closest to ground during normal operation, wherein the mat arrangement comprises a mat attachment arrangement that connects the mat to the body in a movable manner.
- 2. The robotic lawn mower according to claim 1, wherein the mat attachment arrangement comprises a spring-biased holder that is adapted to press the first edge towards ground during normal operation.
- 3. The robotic lawn mower according to claim 1, wherein the mat attachment arrangement comprises a pivotable mat holder that is pivotable along a longitudinally running pivot axis that runs mainly parallel to the first edge, wherein the pivotable mat holder is spring-biased to retain the first edge biased towards ground during normal operation.
- 4. The robotic lawn mower according to claim 1, wherein the mat attachment arrangement comprises a mat holder that is rotably connected to the disc rotation axle such that the mat holder has a vertical position that follows a vertical position of the cutting disc while the first edge is maintained running mainly across the forward running direction.
- 5. The robotic lawn mower according to claim 1, wherein the mat is a resilient mat that comprises a plurality of brush bristles that run between the first edge and a second edge that runs mainly parallel to the first edge.
- 6. The robotic lawn mower according to claim 1, wherein the mat is a resilient mat that comprises a rubber sheet that runs between the first edge and a second edge that runs mainly parallel to the first edge.
- 7. The robotic lawn mower according to claim 1, wherein the mat comprises a plurality of pins that run between the first edge and a second edge that runs mainly parallel to the first edge, wherein the pins are connected to a pin holding rod.
- 8. The robotic lawn mower according to claim 1, wherein the mat is positioned between a drive wheel axis and the rearmost end of the robotic lawn mower.
- 9. The robotic lawn mower according to claim 1, wherein the mat is positioned between a drive wheel axis and the frontmost end of the robotic lawn mower.
- 10. The robotic lawn mower according to claim 1, comprising at least one further mat arrangement.
- 11. The robotic lawn mower according to claim 10, comprising a first mat arrangement and a second mat arrangement, wherein the mat arrangements are positioned between the cutting disc and the rearmost end of the robotic lawn mower.
- 12. The robotic lawn mower according to claim 11, wherein the mat arrangements comprise mutually different types of mats.
- 13. The robotic lawn mower according to claim 12, wherein the first mat arrangement is positioned closer to the rearmost end of the robotic lawn mower than the second mat arrangement, wherein the first mat arrangement comprises a first mat that in turn comprises a plurality of brush bristles that run between the first edge and a second edge that runs mainly parallel to the first edge, and wherein the second mat arrangement comprises a second mat that in turn comprises a plurality of pins that run between the first edge and a second edge that runs mainly parallel to the first edge.
- 14. The robotic lawn mower according to claim 1, wherein the first edge is adapted to reach a maximum distance into the grass that is to be cut, wherein the maximum distance lies between 40% and 60% of the average grass height.
- 15. The robotic lawn mower according to claim 1, wherein the first edge is adapted to be biased towards a grass surface with a force that lies between 5N and 40N.
- 16. The robotic lawn mower according to claim 1, wherein the body has a circumferentially running perimeter that faces ground during normal operation, wherein the mat extends within the perimeter.</t>
-  </si>
-  <si>
     <t>_Terramow - Grass Comb Related Patents.xlsx</t>
   </si>
   <si>
-    <t>US12690517B2</t>
-  </si>
-  <si>
-    <t>Lawn mower</t>
-  </si>
-  <si>
-    <t>A lawn mower comprising a lawn mower body, wherein a cutting chamber is arranged at the bottom of the lawn mower body, a blade is rotatably connected to the middle of the cutting chamber, and a plurality of first grass inlet channels communicated with the cutting chamber are arranged on the front side of the bottom of the lawn mower body, wherein the plurality of first grass inlet channels are provided with a supporting mechanism for improving the total bending resistance of the grass in the cutting process; during the traveling of the lawn mower body, the grass to be cut enters between the plurality of supporting pieces from the first grass inlet channels and the second grass inlet channels of the base of the supporting mechanism, and the top of the grass to be cut passes out from the supporting pieces.</t>
-  </si>
-  <si>
-    <t>1. A lawn mower, comprising: a lawn mower body (1), wherein a cutting chamber (11) is arranged at a bottom of the lawn mower body (1), a blade (12) is rotatably connected to a middle of the cutting chamber (11), and a plurality of first grass inlet channels (13) communicated with the cutting chamber (11) are arranged on a front side of the bottom of the lawn mower body (1), wherein the plurality of first grass inlet channels (13) are provided with a supporting mechanism (2) for improving a total bending resistance of grass during cutting, and the supporting mechanism (2) comprises a base (21) detachably arranged on the plurality of first grass inlet channels (13) and a plurality of supporting pieces (22) arranged side by side on the base (21) and extending to a lower portion of the cutting chamber (11), wherein the base (21) is provided with a plurality of second grass inlet channels (211) respectively communicated with the plurality of first grass inlet channels (13), wherein an orthographic projection of a rotation range of the blade (12) overlaps with orthographic projections of the plurality of supporting pieces (22), wherein along an extension direction of the plurality of first grass inlet channels (13), a length that the orthographic projection of the rotation range of the blade (12) overlaps with the orthographic projections of the plurality of supporting pieces (22) is not less than a ratio of distance S meters travelled by the lawn mower body (1) per second to n revolutions per second of the blade (12).</t>
-  </si>
-  <si>
-    <t>What is claimed is:
- 1. A lawn mower, comprising:
-  a lawn mower body (1), wherein a cutting chamber (11) is arranged at a bottom of the lawn mower body (1), a blade (12) is rotatably connected to a middle of the cutting chamber (11), and a plurality of first grass inlet channels (13) communicated with the cutting chamber (11) are arranged on a front side of the bottom of the lawn mower body (1), wherein the plurality of first grass inlet channels (13) are provided with a supporting mechanism (2) for improving a total bending resistance of grass during cutting, and the supporting mechanism (2) comprises a base (21) detachably arranged on the plurality of first grass inlet channels (13) and a plurality of supporting pieces (22) arranged side by side on the base (21) and extending to a lower portion of the cutting chamber (11), wherein the base (21) is provided with a plurality of second grass inlet channels (211) respectively communicated with the plurality of first grass inlet channels (13), wherein an orthographic projection of a rotation range of the blade (12) overlaps with orthographic projections of the plurality of supporting pieces (22),
-  wherein along an extension direction of the plurality of first grass inlet channels (13), a length that the orthographic projection of the rotation range of the blade (12) overlaps with the orthographic projections of the plurality of supporting pieces (22) is not less than a ratio of distance S meters travelled by the lawn mower body (1) per second to n revolutions per second of the blade (12).
- 2. The lawn mower of claim 1, wherein lengths of the plurality of supporting pieces (22) extending toward the cutting chamber (11) are different, wherein a connecting line of end points of the plurality of support pieces (22) close to one end of the cutting chamber (11) is configured to be arc-shaped, and its center is located on a rotation center line of the blade.
- 3. The lawn mower of claim 1, wherein along the extension direction of the plurality of first grass inlet channels (13), the length that the orthographic projection of the rotation range of the blade (12) overlaps with the orthographic projections of the plurality of support pieces (22) is 10-30 mm.
- 4. The lawn mower of claim 1, wherein a thickness of each of the plurality of supporting pieces (22) is 4-6 mm, and a distance between two adjacent supporting pieces (22) is 30-40 mm.
- 5. The lawn mower of claim 1, wherein a height of each of the plurality of supporting pieces (22) is 10-15 mm.
- 6. The lawn mower of claim 1, wherein a distance between an upper surface of each of the plurality of supporting pieces (22) and the blade (12) is 4-6 mm.
- 7. The lawn mower of claim 1, wherein the base is fixedly connected to the plurality of first grass inlet channels (13) through a plurality of bolts (3).</t>
-  </si>
-  <si>
-    <t>An automated robotic lawn mower system with an interactive user interface that enables users to configure and monitor mowing operations. The system allows users to create and modify no-go zones on a map using finger gestures and can automatically suggest a no-go zone when the mower becomes stuck. Users can adjust various mowing parameters, including cutting height, edge-cutting distance, mowing path spacing, travel speed, blade-disc rotation speed, and mowing direction. The interface also provides visualization of the mower's cutting path for tracking progress and a multi-color visual status indicator that communicates mower operating conditions through different colors and illumination patterns.</t>
-  </si>
-  <si>
-    <t>US12213402B2</t>
-  </si>
-  <si>
-    <t>Robotic work tool system and method for defining a stay-out area within a work area</t>
-  </si>
-  <si>
     <t>H</t>
   </si>
   <si>
-    <t>A robotic work tool system (200) for defining a stay-out area (120) within a work area (150). The stay-out area (120) is an area which is to be excluded from the work area (150) in which a robotic work tool (100) is subsequently intended to operate. The robotic work tool system (200) comprises a boundary definition unit (130) comprising at least one position unit (175) configured to receive position data and at least one controller (110, 210). The controller (110, 210) is configured to receive a stay-out area definition trigger signal, which indicates that the boundary definition unit (130) has approached the stay-out area to be defined. The controller (110, 210) is further configured to receive, based on the received signal, position data indicating the present position of the boundary definition unit (130) from the position unit (175). The controller (110, 210) is further configured to define the stay-out area (120) as an area centered at an offset from the received position data.</t>
-  </si>
-  <si>
-    <t>1. A robotic work tool system for defining a stay-out area within a work area, wherein the stay-out area is an area which is to be excluded from the work area in which a boundary definition unit is intended to operate, the robotic work tool system comprising:the boundary definition unit comprising a position unit configured to receive position data;a controller configured to:receive a stay-out area definition trigger signal, wherein the stay-out area definition trigger signal is a signal that indicates that the boundary definition unit has approached the stay-out area to be defined;receive, based on the received stay-out area definition trigger signal, position data from the position unit, wherein the position data indicates a present position of the boundary definition unit; anddefine the stay-out area as an area centered at an offset from the received position data.20. A method performed by a robotic work tool system for defining a stay-out area within a work area, wherein the stay-out area is an area which is to be excluded from the work area in which a robotic work tool is intended to operate, wherein the method comprises:receiving a stay-out area definition trigger signal, wherein the stay-out area definition trigger signal is a signal that indicates that a boundary definition unit has approached the stay-out area to be defined;receiving, based on the received stay-out area definition trigger signal, position data, wherein the position data indicates the present position of the boundary definition unit; anddefining the stay-out area as an area centered at an offset from the received position data.</t>
-  </si>
-  <si>
-    <t>The invention claimed is:1. A robotic work tool system for defining a stay-out area within a work area, wherein the stay-out area is an area which is to be excluded from the work area in which a boundary definition unit is intended to operate, the robotic work tool system comprising: the boundary definition unit comprising a position unit configured to receive position data; a controller configured to: receive a stay-out area definition trigger signal, wherein the stay-out area definition trigger signal is a signal that indicates that the boundary definition unit has approached the stay-out area to be defined; receive, based on the received stay-out area definition trigger signal, position data from the position unit, wherein the position data indicates a present position of the boundary definition unit; and define the stay-out area as an area centered at an offset from the received position data.2. The robotic work tool system according to claim 1, wherein the controller is configured to position an outer perimeter of the stay-out area at the present position of the boundary definition unit.3. The robotic work tool system according to claim 1, wherein said offset comprises an offset direction.4. The robotic work tool system according to claim 3, wherein said offset direction is based on a heading of the boundary definition unit.5. The robotic work tool system according to claim 1, wherein said offset comprises an offset distance.6. The robotic work tool system according to claim 5, wherein said offset distance is set based on a size of the stay-out area.7. The robotic work tool system according to claim 1, wherein said offset is a predefined offset.8. The robotic work tool system according to claim 1, wherein the robotic work tool system further comprises a user interface configured to receive user input from a user during the user's operation and interaction with said user interface, wherein the user interface is configured to receive input related to the stay-out area.9. The robotic work tool system according to claim 8, wherein the controller further is configured to define the stay-out area based on the received user input.10. The robotic work tool system according to claim 9, wherein said offset comprises an offset distance that is adjustable via the user interface and the received user input determines the offset distance.11. The robotic work tool system according to claim 9, wherein the received user input determines a shape of the stay-out area.12. The robotic work tool system according to claim 11, wherein the shape of the stay-out area is selectable from a set of predefined shapes in the user interface.13. The robotic work tool system according to claim 12, wherein the shape of the stay-out area is at least one from a group comprising: a circle, a square and a rectangle.14. The robotic work tool system according to claim 11, wherein an orientation of the shape of the stay-out area is adjustable via the user interface and the received user input determines the orientation of the shape of the stay-out area.15. The robotic work tool system according to claim 11, wherein an aspect ratio of the shape of the stay-out area is adjustable via the user interface and the received user input determines the aspect ratio of the shape of the stay-out area.16. The robotic work tool system according to claim 8, wherein the stay-out area definition trigger signal is based on input received via the user interface.17. The robotic work tool system according to claim 1, wherein the boundary definition unit further comprises a sensor unit configured to receive sensor data indicating that an object is located in front of the boundary definition unit and wherein the stay-out area definition trigger signal is based on the received sensor data.18. The robotic work tool system according to claim 1, wherein the stay-out area definition trigger signal is based on a signal indicating that the boundary definition unit is not moving, and wherein the signal indicating that the boundary definition unit is not moving is received from at least one from a group comprising: a motor, an odometer and an accelerometer.19. The robotic work tool system according to claim 1, wherein the boundary definition unit is a robotic work tool, and the robotic work tool is a robotic lawn mower.20. A method performed by a robotic work tool system for defining a stay-out area within a work area, wherein the stay-out area is an area which is to be excluded from the work area in which a robotic work tool is intended to operate, wherein the method comprises: receiving a stay-out area definition trigger signal, wherein the stay-out area definition trigger signal is a signal that indicates that a boundary definition unit has approached the stay-out area to be defined; receiving, based on the received stay-out area definition trigger signal, position data, wherein the position data indicates the present position of the boundary definition unit; and defining the stay-out area as an area centered at an offset from the received position data.</t>
-  </si>
-  <si>
     <t>Terramow UI - Mowing Settings Related Patents.xlsx</t>
-  </si>
-  <si>
-    <t>US9475196B2</t>
-  </si>
-  <si>
-    <t>Detachable user interface for a robotic vehicle</t>
-  </si>
-  <si>
-    <t>A robotic vehicle may include control circuitry, a device interface and a detachable user interface. The control circuitry may be configured to execute stored instructions to direct operation of the robotic vehicle on a defined area. The device interface may enable electronic communication of a device with the control circuitry. The detachable user interface may be configured to be removably mated with the robotic vehicle to enable communication between the detachable user interface and the control circuitry via the device interface. The detachable user interface may provide user interface capability to enable an operator to define one or more setting parameters or instructions responsive to the detachable user interface being mated with the robotic vehicle for execution by the control circuitry to control operation of the robotic vehicle when the detachable user interface is not mated with the robotic vehicle.</t>
-  </si>
-  <si>
-    <t>1. A robotic vehicle comprising: control circuitry configured to execute stored instructions to direct operation of the robotic vehicle on a defined area; a device interface enabling electronic communication between one or more devices and the control circuitry; and a detachable user interface configured to be removably mated with the robotic vehicle to enable communication between the detachable user interface and the control circuitry via the device interface, the detachable user interface providing user interface capability to enable an operator to define one or more setting parameters or instructions responsive to the detachable user interface being mated with the robotic vehicle for execution by the control circuitry to control operation of the robotic vehicle when the detachable user interface is not mated with the robotic vehicle, wherein being mated comprises at least a portion of a detachable user interface housing being received within a docking station of the detachable user interface.10. A detachable user interface comprising processing circuitry configured to interface with control circuitry of a robotic vehicle responsive to mating of the detachable user interface with the robotic vehicle via a device interface of the robotic vehicle, wherein the control circuitry is configured to execute stored instructions to direct operation of the robotic vehicle on a defined area, and wherein the detachable user interface is configured to be removably mated with the robotic vehicle to enable communication between the detachable user interface and the control circuitry via the device interface, the detachable user interface providing user interface capability to enable an operator to define one or more setting parameters or instructions responsive to the detachable user interface being mated with the robotic vehicle for execution by the control circuitry to control operation of the robotic vehicle when the detachable user interface is not mated with the robotic vehicle, wherein being mated comprises at least a portion of a detachable user interface housing being received within a docking station of the detachable user interface.</t>
-  </si>
-  <si>
-    <t>That which is claimed:1. A robotic vehicle comprising: control circuitry configured to execute stored instructions to direct operation of the robotic vehicle on a defined area; a device interface enabling electronic communication between one or more devices and the control circuitry; and a detachable user interface configured to be removably mated with the robotic vehicle to enable communication between the detachable user interface and the control circuitry via the device interface, the detachable user interface providing user interface capability to enable an operator to define one or more setting parameters or instructions responsive to the detachable user interface being mated with the robotic vehicle for execution by the control circuitry to control operation of the robotic vehicle when the detachable user interface is not mated with the robotic vehicle, wherein being mated comprises at least a portion of a detachable user interface housing being received within a docking station of the detachable user interface.2. The robotic vehicle of claim 1, wherein the docking station includes one or more electrical contacts configured to electrically mate with one or more electrical contacts of the detachable user interface responsive to insertion of the detachable user interface into the docking station.3. The robotic vehicle of claim 1, wherein the docking station includes a wireless communication mechanism for interfacing with the detachable user interface responsive to insertion of the detachable user interface into the docking station.4. The robotic vehicle of claim 3, wherein the wireless communication mechanism employs voice recognition technology.5. The robotic vehicle of claim 1, wherein the detachable user interface includes a display.6. The robotic vehicle of claim 1, wherein the detachable user interface is powered from the robotic vehicle or includes an onboard power supply.7. The robotic vehicle of claim 1, wherein the detachable user interface includes a casing configured to snap fit with a housing of the robotic vehicle.8. The robotic vehicle of claim 7, wherein the robotic vehicle includes retractable detents biased to engage the casing, rotatable levers, or magnets to hold the detachable user interface to the robotic vehicle.9. The robotic vehicle of claim 1, wherein the communication of setting parameters or instructions to the control circuitry is enabled responsive to entry of a code pairing the detachable user interface with the control circuitry.10. A detachable user interface comprising processing circuitry configured to interface with control circuitry of a robotic vehicle responsive to mating of the detachable user interface with the robotic vehicle via a device interface of the robotic vehicle, wherein the control circuitry is configured to execute stored instructions to direct operation of the robotic vehicle on a defined area, and wherein the detachable user interface is configured to be removably mated with the robotic vehicle to enable communication between the detachable user interface and the control circuitry via the device interface, the detachable user interface providing user interface capability to enable an operator to define one or more setting parameters or instructions responsive to the detachable user interface being mated with the robotic vehicle for execution by the control circuitry to control operation of the robotic vehicle when the detachable user interface is not mated with the robotic vehicle, wherein being mated comprises at least a portion of a detachable user interface housing being received within a docking station of the detachable user interface.11. The detachable user interface of claim 10, wherein the detachable user interface includes one or more electrical contacts configured to electrically mate with one or more electrical contacts of the docking station responsive to insertion of the detachable user interface into the docking station.12. The detachable user interface of claim 10, wherein the detachable user interface includes a wireless communication mechanism for interfacing with the docking station responsive to insertion of the detachable user interface into the docking station.13. The detachable user interface of claim 12, wherein the wireless communication mechanism employs voice recognition technology.14. The detachable user interface of claim 10, wherein the detachable user interface includes a display.15. The detachable user interface of claim 10, wherein the detachable user interface is powered from the robotic vehicle.16. The detachable user interface of claim 10, wherein the detachable user interface includes a casing configured to snap fit with a housing of the robotic vehicle.17. The detachable user interface of claim 16, wherein the robotic vehicle includes retractable detents biased to engage the casing, rotatable levers, or magnets to hold the detachable user interface to the robotic vehicle.18. The detachable user interface of claim 10, wherein the communication of setting parameters or instructions to the control circuitry is enabled responsive to entry of a code pairing the detachable user interface with the control circuitry.</t>
   </si>
   <si>
     <t>An automated robotic lawn mower incorporating rain detection and a replaceable battery system. The mower uses a rain sensor to detect rainfall and automatically return to a base station, with the capability to resume mowing once the grass has dried. The mower further includes a removable battery assembly accessible from the bottom of the mower body, housed in a battery compartment with a removable battery cover and screw-secured inner cover. The battery is equipped with a handle and electrical connector to facilitate convenient removal, replacement, and electrical connection of the battery.</t>
@@ -406,34 +313,6 @@
     <t>Blower – Variable Pitch Fan Blade Noise Reduction Related Patents.xlsx</t>
   </si>
   <si>
-    <t>CN210371324U</t>
-  </si>
-  <si>
-    <t>High/efficiency low/noise fan blade</t>
-  </si>
-  <si>
-    <t>The utility model discloses a high/efficiency low/noise fan blade which comprises an air protection ring, blades and a hub. The seven blades are distributed along the periphery of the hub at unequal intervals; each blade is in the shape of a bird wing, is of a forward/bent sweepback structure and is obliquely mounted; the bending angle of the blade from the blade root to the blade middle is increased from 0 degree to 9/10 degrees, and the bending angle of the blade from the blade middle to the blade top is decreased from/9 degrees to/10 degrees; the inclination angle of the blade from the blade root to the middle part of the blade is decreased from 24/25 degrees to 15/16 degrees, and the inclination angle of the blade from the middle part of the blade to the blade top is increased from 17/18 degrees; and from the blade root to the blade top, the ratio of the chord length of the radius section of the blade to the mounting radius is gradually reduced from 0.7/0.8 to 0.30/0.31. Under thecondition that the flow performance of an existing product is met, the blade profile camber, the chord length, the blade surface and the like are optimized, the sound quality is improved, and the structural strength of the fan blade is improved.</t>
-  </si>
-  <si>
-    <t>1. A high/efficiency low/noise fan blade comprises a wind protection ring, a blade and a hub, wherein the blade is connected with the wind protection ring at the blade top and is connected with the hub at the blade root; the method is characterized in that:the blades are distributed along the periphery of the hub in unequal intervals, the size of an included angle formed by connecting lines of the middle points of the blade roots of the adjacent blades and the center of the hub is used as an interval angle, the blades are marked by self/turning, and the interval angles of the adjacent blades are 55/57 degrees, 49/51 degrees, 52/54 degrees, 44/46 degrees, 58/60 degrees, 46/48 degrees and 49/51 degrees in sequence along the running direction;each blade is in a bird wing shape, is in a forward/bending and backward/sweeping structure and is obliquely installed;the included angle formed by the connecting line of the front edge of each position of the blade and the center of the hub and the connecting line of the front edge of the blade and the center of the hub is taken as the bending angle of each position, the reverse direction of the running direction is taken as the positive direction, the bending angle from the blade root to the middle part of the blade is gradually increased from 0 degree to 9/10 degrees, and the bending angle from the middle part of the blade to the blade top is gradually decreased to/9/10 degrees;the section of each blade parallel to the cylindrical surface of the hub is taken as a radius section, the connecting line of the front edge and the rear edge of the radius section is taken as a chord length line of the radius section, and the included angle between the chord length line of the radius section at each position of the blade and the hub surface is taken as an inclination angle; the inclination angle from the blade root to the middle part of the blade is gradually decreased from 24/25 degrees to 15/16 degrees, and the inclination angle from the middle part of the blade to the blade top is gradually increased to 17/18 degrees;the distance from each position of the blade to the center of the hub is taken as an installation radius, and the ratio of the chord length of the section of the radius to the installation radius gradually decreases from 0.7/0.8 to 0.30/0.31 from the blade root to the blade top.</t>
-  </si>
-  <si>
-    <t>1. A high/efficiency low/noise fan blade comprises a wind protection ring, a blade and a hub, wherein the blade is connected with the wind protection ring at the blade top and is connected with the hub at the blade root; the method is characterized in that:
- the blades are distributed along the periphery of the hub in unequal intervals, the size of an included angle formed by connecting lines of the middle points of the blade roots of the adjacent blades and the center of the hub is used as an interval angle, the blades are marked by self/turning, and the interval angles of the adjacent blades are 55/57 degrees, 49/51 degrees, 52/54 degrees, 44/46 degrees, 58/60 degrees, 46/48 degrees and 49/51 degrees in sequence along the running direction;
- each blade is in a bird wing shape, is in a forward/bending and backward/sweeping structure and is obliquely installed;
- the included angle formed by the connecting line of the front edge of each position of the blade and the center of the hub and the connecting line of the front edge of the blade and the center of the hub is taken as the bending angle of each position, the reverse direction of the running direction is taken as the positive direction, the bending angle from the blade root to the middle part of the blade is gradually increased from 0 degree to 9/10 degrees, and the bending angle from the middle part of the blade to the blade top is gradually decreased to/9/10 degrees;
- the section of each blade parallel to the cylindrical surface of the hub is taken as a radius section, the connecting line of the front edge and the rear edge of the radius section is taken as a chord length line of the radius section, and the included angle between the chord length line of the radius section at each position of the blade and the hub surface is taken as an inclination angle; the inclination angle from the blade root to the middle part of the blade is gradually decreased from 24/25 degrees to 15/16 degrees, and the inclination angle from the middle part of the blade to the blade top is gradually increased to 17/18 degrees;
- the distance from each position of the blade to the center of the hub is taken as an installation radius, and the ratio of the chord length of the section of the radius to the installation radius gradually decreases from 0.7/0.8 to 0.30/0.31 from the blade root to the blade top.
- 2. The high efficiency, low noise fan blade of claim 1 wherein the spacing angles between adjacent blades, as measured from the direction of rotation marking the blade start, are in turn 56 °, 50 °, 53 °, 45 °, 60 °, 48 °, 49 °.
- 3. The high/efficiency low/noise fan blade as claimed in claim 1, wherein the bending angles of the blades at 11 equally spaced radius sections from the blade root to the blade top are 0 °, 4/5 °, 6/7 °, 7/8 °, 8/9 °, 7/8 °, 4/5 °, 2/3 °, 3/2 ° and/9/8 ° in sequence.
- 4. The high/efficiency low/noise fan blade as claimed in claim 1, wherein the inclination angles of the equally spaced 11 radius sections of each fan blade from the blade root to the blade top are 24/25 °, 21/22 °, 19/20 °, 17/18 °, 16/17 °, 15/16 °, 16/17 ° and 17/18 ° in sequence.
- 5. The high efficiency low noise blade of claim 1 wherein each blade has a ratio of radial cross/sectional chord length to mounting radius of 0.78, 0.67, 0.576, 0.512, 0.461, 0.412, 0.379, 0.345, 0.324, 0.318, 0.308 from blade root to blade tip.
- 6. A high efficiency, low noise wind blade according to claim 1 wherein the radial cross section of the blade is an aerofoil cross section.
- 7. The high efficiency low noise fan blade of claim 1 wherein said hub has a circumferentially inwardly recessed annular structure near the periphery thereof.
- 8. The high efficiency low noise fan blade of claim 1 wherein said hub surface is slotted.
- 9. The high efficiency, low noise fan blade of claim 1 wherein said shroud ring, blade and hub are of unitary injection molded construction.</t>
-  </si>
-  <si>
     <t>Suncut lotion / sunscreen cosmetic composition</t>
   </si>
   <si>
@@ -630,12 +509,15 @@
   <si>
     <t>Total</t>
   </si>
+  <si>
+    <t>title</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -648,6 +530,18 @@
       <sz val="11"/>
       <name val="Cambria"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Cambria"/>
+      <family val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -685,7 +579,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -696,7 +590,11 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
   </cellXfs>
@@ -895,7 +793,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -905,427 +803,263 @@
     <col min="5" max="5" width="65" customWidth="1"/>
     <col min="6" max="6" width="80" customWidth="1"/>
     <col min="7" max="7" width="100" customWidth="1"/>
-    <col min="8" max="8" width="55" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="D1" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="E1" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="3" t="s">
+      <c r="F1" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="G1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="H1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="4" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="4" t="s">
+      <c r="B2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="C2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="D2" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="F2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="H2" s="4" t="s">
+    </row>
+    <row r="3" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" s="4" t="s">
         <v>15</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="4" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" s="4" t="s">
+      <c r="C3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="E3" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="F3" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+    </row>
+    <row r="4" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" s="4" t="s">
+      <c r="E4" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="H4" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="4" t="s">
+      <c r="B5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>38</v>
+      </c>
+      <c r="D6" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>35</v>
-      </c>
-      <c r="C6" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>37</v>
-      </c>
       <c r="E6" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="H6" s="4" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C7" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="G7" s="4" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
-        <v>47</v>
-      </c>
       <c r="B8" s="4" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>47</v>
+        <v>55</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C9" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="G9" s="4" t="s">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="D9" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>57</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>58</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="4" t="s">
-        <v>59</v>
-      </c>
       <c r="B10" s="4" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>37</v>
+        <v>10</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G10" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" s="5" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>59</v>
+        <v>55</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>11</v>
+        <v>17</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="G11" s="4" t="s">
-        <v>70</v>
-      </c>
-      <c r="H11" s="4" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="4" t="s">
         <v>71</v>
       </c>
-      <c r="B12" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="C12" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>78</v>
-      </c>
-      <c r="C13" s="4" t="s">
-        <v>79</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>81</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A14" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>85</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>86</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>88</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A15" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>90</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>92</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
-        <v>83</v>
-      </c>
-      <c r="B16" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>96</v>
-      </c>
-      <c r="D16" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="E16" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>98</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="H16" s="4" t="s">
-        <v>89</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H36" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:G31" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
@@ -1342,21 +1076,21 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="2" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>65</v>
+        <v>42</v>
       </c>
       <c r="B2" s="2">
         <v>1</v>
@@ -1370,7 +1104,7 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>89</v>
+        <v>61</v>
       </c>
       <c r="B3" s="2">
         <v>1</v>
@@ -1384,7 +1118,7 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>77</v>
+        <v>49</v>
       </c>
       <c r="B4" s="2">
         <v>1</v>
@@ -1398,7 +1132,7 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="B5" s="2">
         <v>1</v>
@@ -1412,7 +1146,7 @@
     </row>
     <row r="6" spans="1:4" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
-        <v>53</v>
+        <v>30</v>
       </c>
       <c r="B6" s="2">
         <v>1</v>
@@ -1426,7 +1160,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A7" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B7" s="2">
         <v>0</v>
@@ -1440,7 +1174,7 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A8" s="2" t="s">
-        <v>28</v>
+        <v>21</v>
       </c>
       <c r="B8" s="2">
         <v>0</v>
@@ -1470,15 +1204,15 @@
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>100</v>
+        <v>72</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
-        <v>37</v>
+        <v>22</v>
       </c>
       <c r="B2" s="2">
         <v>5</v>
@@ -1486,7 +1220,7 @@
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B3" s="2">
         <v>5</v>
@@ -1494,7 +1228,7 @@
     </row>
     <row r="4" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B4" s="2">
         <v>5</v>
@@ -1502,7 +1236,7 @@
     </row>
     <row r="5" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
-        <v>101</v>
+        <v>73</v>
       </c>
       <c r="B5" s="2">
         <v>15</v>

</xml_diff>